<commit_message>
Changed findings weight in excel file
</commit_message>
<xml_diff>
--- a/Costing-Format_5_formats.xlsx
+++ b/Costing-Format_5_formats.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project_Files\Sushil_Sir\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\INTERNGOLD_PROJECTS\sushil_sir_style_breakup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{69C42C7D-844A-4178-A2FA-6DC4320D8C4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E0C4A21-8E80-413B-8624-A5526FEA9001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="953" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -820,7 +820,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A316E669-1616-44D9-AE44-E0264B4E3C0F}">
-  <dimension ref="A1:XFD60"/>
+  <dimension ref="A1:XFD50"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.5546875" style="1" customWidth="1"/>
@@ -1123,7 +1123,7 @@
       <c r="AP4" s="29"/>
       <c r="XFD4" s="1"/>
     </row>
-    <row r="5" spans="1:42 16384:16384" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:42 16384:16384" x14ac:dyDescent="0.3">
       <c r="A5" s="10">
         <v>1</v>
       </c>
@@ -1153,7 +1153,7 @@
         <v>75</v>
       </c>
       <c r="K5" s="5">
-        <f>J5/31.1035*E5/0.9*I5</f>
+        <f>J5/31.1035*E5/0.85*I5</f>
         <v>0</v>
       </c>
       <c r="L5" s="31"/>
@@ -1247,7 +1247,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="6" spans="1:42 16384:16384" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:42 16384:16384" x14ac:dyDescent="0.3">
       <c r="A6" s="10"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -1337,7 +1337,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="7" spans="1:42 16384:16384" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:42 16384:16384" x14ac:dyDescent="0.3">
       <c r="A7" s="10"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -1427,7 +1427,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="8" spans="1:42 16384:16384" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:42 16384:16384" x14ac:dyDescent="0.3">
       <c r="A8" s="10"/>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -1517,7 +1517,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="9" spans="1:42 16384:16384" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:42 16384:16384" x14ac:dyDescent="0.3">
       <c r="A9" s="10"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -1607,7 +1607,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="10" spans="1:42 16384:16384" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:42 16384:16384" x14ac:dyDescent="0.3">
       <c r="A10" s="10"/>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -1649,9 +1649,8 @@
       <c r="AM10" s="10"/>
       <c r="AN10" s="13"/>
       <c r="AO10" s="10"/>
-      <c r="AP10" s="28"/>
-    </row>
-    <row r="11" spans="1:42 16384:16384" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:42 16384:16384" x14ac:dyDescent="0.3">
       <c r="A11" s="10"/>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -1693,9 +1692,8 @@
       <c r="AM11" s="10"/>
       <c r="AN11" s="13"/>
       <c r="AO11" s="10"/>
-      <c r="AP11" s="28"/>
-    </row>
-    <row r="12" spans="1:42 16384:16384" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:42 16384:16384" x14ac:dyDescent="0.3">
       <c r="A12" s="10"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -1737,9 +1735,8 @@
       <c r="AM12" s="10"/>
       <c r="AN12" s="13"/>
       <c r="AO12" s="10"/>
-      <c r="AP12" s="28"/>
-    </row>
-    <row r="13" spans="1:42 16384:16384" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:42 16384:16384" x14ac:dyDescent="0.3">
       <c r="A13" s="10"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -1781,9 +1778,8 @@
       <c r="AM13" s="10"/>
       <c r="AN13" s="13"/>
       <c r="AO13" s="10"/>
-      <c r="AP13" s="28"/>
-    </row>
-    <row r="14" spans="1:42 16384:16384" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:42 16384:16384" x14ac:dyDescent="0.3">
       <c r="A14" s="10">
         <v>2</v>
       </c>
@@ -1907,7 +1903,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="15" spans="1:42 16384:16384" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:42 16384:16384" x14ac:dyDescent="0.3">
       <c r="A15" s="10"/>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
@@ -1997,7 +1993,7 @@
         <v>0.21999999999999997</v>
       </c>
     </row>
-    <row r="16" spans="1:42 16384:16384" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:42 16384:16384" x14ac:dyDescent="0.3">
       <c r="A16" s="10"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -2087,7 +2083,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="17" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A17" s="10"/>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
@@ -2177,7 +2173,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="18" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A18" s="10"/>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
@@ -2267,7 +2263,7 @@
         <v>0.21999999999999995</v>
       </c>
     </row>
-    <row r="19" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A19" s="10"/>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
@@ -2309,9 +2305,8 @@
       <c r="AM19" s="10"/>
       <c r="AN19" s="13"/>
       <c r="AO19" s="10"/>
-      <c r="AP19" s="28"/>
-    </row>
-    <row r="20" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A20" s="10"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
@@ -2355,9 +2350,8 @@
       <c r="AM20" s="10"/>
       <c r="AN20" s="13"/>
       <c r="AO20" s="10"/>
-      <c r="AP20" s="28"/>
-    </row>
-    <row r="21" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A21" s="10"/>
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
@@ -2399,9 +2393,8 @@
       <c r="AM21" s="10"/>
       <c r="AN21" s="13"/>
       <c r="AO21" s="10"/>
-      <c r="AP21" s="28"/>
-    </row>
-    <row r="22" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A22" s="10"/>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
@@ -2443,9 +2436,8 @@
       <c r="AM22" s="10"/>
       <c r="AN22" s="13"/>
       <c r="AO22" s="10"/>
-      <c r="AP22" s="28"/>
-    </row>
-    <row r="23" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A23" s="10">
         <v>3</v>
       </c>
@@ -2569,7 +2561,7 @@
         <v>0.21999999999999989</v>
       </c>
     </row>
-    <row r="24" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A24" s="10"/>
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
@@ -2585,18 +2577,18 @@
         <v>0</v>
       </c>
       <c r="H24" s="15">
-        <v>1.1499999999999999</v>
+        <v>1</v>
       </c>
       <c r="I24" s="15">
         <f>G24+H24</f>
-        <v>1.1499999999999999</v>
+        <v>1</v>
       </c>
       <c r="J24" s="5">
         <v>4500</v>
       </c>
       <c r="K24" s="5">
         <f>J24/31.1035/24*E24/0.9*I24</f>
-        <v>69.324995579275651</v>
+        <v>60.282604851544043</v>
       </c>
       <c r="L24" s="31"/>
       <c r="M24" s="35"/>
@@ -2644,22 +2636,22 @@
       </c>
       <c r="AM24" s="5">
         <f>(K24+Y23+AH24+AI24+AJ24+AK24+AL24)</f>
-        <v>85.324995579275651</v>
+        <v>76.28260485154405</v>
       </c>
       <c r="AN24" s="4">
         <f>AM24/0.78</f>
-        <v>109.39101997343032</v>
+        <v>97.798211348133393</v>
       </c>
       <c r="AO24" s="17">
         <f>CEILING(AN24,1)</f>
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="AP24" s="28">
         <f>(AN24-AM24)/AN24</f>
-        <v>0.21999999999999997</v>
-      </c>
-    </row>
-    <row r="25" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+        <v>0.21999999999999995</v>
+      </c>
+    </row>
+    <row r="25" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A25" s="10"/>
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
@@ -2749,7 +2741,7 @@
         <v>0.21999999999999992</v>
       </c>
     </row>
-    <row r="26" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A26" s="10"/>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
@@ -2839,7 +2831,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="27" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A27" s="10"/>
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
@@ -2929,7 +2921,7 @@
         <v>0.21999999999999997</v>
       </c>
     </row>
-    <row r="28" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A28" s="10"/>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
@@ -2971,9 +2963,8 @@
       <c r="AM28" s="10"/>
       <c r="AN28" s="13"/>
       <c r="AO28" s="10"/>
-      <c r="AP28" s="28"/>
-    </row>
-    <row r="29" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="29" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A29" s="10"/>
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
@@ -3017,9 +3008,8 @@
       <c r="AM29" s="10"/>
       <c r="AN29" s="13"/>
       <c r="AO29" s="10"/>
-      <c r="AP29" s="28"/>
-    </row>
-    <row r="30" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="30" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A30" s="10"/>
       <c r="B30" s="10"/>
       <c r="C30" s="10"/>
@@ -3061,9 +3051,8 @@
       <c r="AM30" s="10"/>
       <c r="AN30" s="13"/>
       <c r="AO30" s="10"/>
-      <c r="AP30" s="28"/>
-    </row>
-    <row r="31" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="31" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A31" s="10"/>
       <c r="B31" s="10"/>
       <c r="C31" s="10"/>
@@ -3105,9 +3094,8 @@
       <c r="AM31" s="10"/>
       <c r="AN31" s="13"/>
       <c r="AO31" s="10"/>
-      <c r="AP31" s="28"/>
-    </row>
-    <row r="32" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="32" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A32" s="10">
         <v>4</v>
       </c>
@@ -3231,7 +3219,7 @@
         <v>0.21999999999999989</v>
       </c>
     </row>
-    <row r="33" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A33" s="10"/>
       <c r="B33" s="10"/>
       <c r="C33" s="10"/>
@@ -3247,18 +3235,18 @@
         <v>0</v>
       </c>
       <c r="H33" s="15">
-        <v>1.1499999999999999</v>
+        <v>1</v>
       </c>
       <c r="I33" s="15">
         <f>G33+H33</f>
-        <v>1.1499999999999999</v>
+        <v>1</v>
       </c>
       <c r="J33" s="5">
         <v>4500</v>
       </c>
       <c r="K33" s="5">
         <f>J33/31.1035/24*E33/0.9*I33</f>
-        <v>69.324995579275651</v>
+        <v>60.282604851544043</v>
       </c>
       <c r="L33" s="31"/>
       <c r="M33" s="35"/>
@@ -3306,22 +3294,22 @@
       </c>
       <c r="AM33" s="5">
         <f>(K33+Y32+AH33+AI33+AJ33+AK33+AL33)</f>
-        <v>85.324995579275651</v>
+        <v>76.28260485154405</v>
       </c>
       <c r="AN33" s="4">
         <f>AM33/0.78</f>
-        <v>109.39101997343032</v>
+        <v>97.798211348133393</v>
       </c>
       <c r="AO33" s="17">
         <f>CEILING(AN33,1)</f>
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="AP33" s="28">
         <f>(AN33-AM33)/AN33</f>
-        <v>0.21999999999999997</v>
-      </c>
-    </row>
-    <row r="34" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+        <v>0.21999999999999995</v>
+      </c>
+    </row>
+    <row r="34" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A34" s="10"/>
       <c r="B34" s="10"/>
       <c r="C34" s="10"/>
@@ -3411,7 +3399,7 @@
         <v>0.21999999999999992</v>
       </c>
     </row>
-    <row r="35" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A35" s="10"/>
       <c r="B35" s="10"/>
       <c r="C35" s="10"/>
@@ -3501,7 +3489,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="36" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A36" s="10"/>
       <c r="B36" s="10"/>
       <c r="C36" s="10"/>
@@ -3591,7 +3579,7 @@
         <v>0.21999999999999997</v>
       </c>
     </row>
-    <row r="37" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A37" s="10"/>
       <c r="B37" s="10"/>
       <c r="C37" s="10"/>
@@ -3633,9 +3621,8 @@
       <c r="AM37" s="10"/>
       <c r="AN37" s="13"/>
       <c r="AO37" s="10"/>
-      <c r="AP37" s="28"/>
-    </row>
-    <row r="38" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="38" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A38" s="10"/>
       <c r="B38" s="10"/>
       <c r="C38" s="10"/>
@@ -3679,9 +3666,8 @@
       <c r="AM38" s="10"/>
       <c r="AN38" s="13"/>
       <c r="AO38" s="10"/>
-      <c r="AP38" s="28"/>
-    </row>
-    <row r="39" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="39" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A39" s="10"/>
       <c r="B39" s="10"/>
       <c r="C39" s="10"/>
@@ -3723,9 +3709,8 @@
       <c r="AM39" s="10"/>
       <c r="AN39" s="13"/>
       <c r="AO39" s="10"/>
-      <c r="AP39" s="28"/>
-    </row>
-    <row r="40" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="40" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A40" s="10"/>
       <c r="B40" s="10"/>
       <c r="C40" s="10"/>
@@ -3767,9 +3752,8 @@
       <c r="AM40" s="10"/>
       <c r="AN40" s="13"/>
       <c r="AO40" s="10"/>
-      <c r="AP40" s="28"/>
-    </row>
-    <row r="41" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="41" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A41" s="10">
         <v>5</v>
       </c>
@@ -3893,7 +3877,7 @@
         <v>0.21999999999999997</v>
       </c>
     </row>
-    <row r="42" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A42" s="10"/>
       <c r="B42" s="10"/>
       <c r="C42" s="10"/>
@@ -3983,7 +3967,7 @@
         <v>0.21999999999999997</v>
       </c>
     </row>
-    <row r="43" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A43" s="10"/>
       <c r="B43" s="10"/>
       <c r="C43" s="10"/>
@@ -4073,7 +4057,7 @@
         <v>0.21999999999999995</v>
       </c>
     </row>
-    <row r="44" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A44" s="10"/>
       <c r="B44" s="10"/>
       <c r="C44" s="10"/>
@@ -4163,7 +4147,7 @@
         <v>0.21999999999999997</v>
       </c>
     </row>
-    <row r="45" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A45" s="10"/>
       <c r="B45" s="10"/>
       <c r="C45" s="10"/>
@@ -4253,7 +4237,7 @@
         <v>0.21999999999999997</v>
       </c>
     </row>
-    <row r="46" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A46" s="10"/>
       <c r="B46" s="10"/>
       <c r="C46" s="10"/>
@@ -4295,9 +4279,8 @@
       <c r="AM46" s="10"/>
       <c r="AN46" s="13"/>
       <c r="AO46" s="10"/>
-      <c r="AP46" s="28"/>
-    </row>
-    <row r="47" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="47" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A47" s="10"/>
       <c r="B47" s="10"/>
       <c r="C47" s="10"/>
@@ -4339,9 +4322,8 @@
       <c r="AM47" s="10"/>
       <c r="AN47" s="13"/>
       <c r="AO47" s="10"/>
-      <c r="AP47" s="28"/>
-    </row>
-    <row r="48" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="48" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A48" s="10"/>
       <c r="B48" s="10"/>
       <c r="C48" s="10"/>
@@ -4385,9 +4367,8 @@
       <c r="AM48" s="10"/>
       <c r="AN48" s="13"/>
       <c r="AO48" s="10"/>
-      <c r="AP48" s="28"/>
-    </row>
-    <row r="49" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="49" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A49" s="10"/>
       <c r="B49" s="10"/>
       <c r="C49" s="10"/>
@@ -4429,9 +4410,8 @@
       <c r="AM49" s="10"/>
       <c r="AN49" s="13"/>
       <c r="AO49" s="10"/>
-      <c r="AP49" s="28"/>
-    </row>
-    <row r="50" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="50" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A50" s="10" t="s">
         <v>39</v>
       </c>
@@ -4475,167 +4455,6 @@
       <c r="AM50" s="10"/>
       <c r="AN50" s="13"/>
       <c r="AO50" s="10"/>
-      <c r="AP50" s="28"/>
-    </row>
-    <row r="51" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="D51" s="25"/>
-      <c r="L51" s="33"/>
-      <c r="M51" s="37"/>
-      <c r="N51" s="40"/>
-      <c r="P51" s="40"/>
-      <c r="Q51" s="45"/>
-      <c r="R51" s="26"/>
-      <c r="S51" s="26"/>
-      <c r="T51" s="26"/>
-      <c r="V51" s="3"/>
-      <c r="X51" s="3"/>
-      <c r="Z51" s="40"/>
-      <c r="AN51" s="3"/>
-      <c r="AP51" s="28"/>
-    </row>
-    <row r="52" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="D52" s="25"/>
-      <c r="L52" s="33"/>
-      <c r="M52" s="37"/>
-      <c r="N52" s="40"/>
-      <c r="P52" s="40"/>
-      <c r="Q52" s="45"/>
-      <c r="R52" s="26"/>
-      <c r="S52" s="26"/>
-      <c r="T52" s="26"/>
-      <c r="V52" s="3"/>
-      <c r="X52" s="3"/>
-      <c r="Z52" s="40"/>
-      <c r="AN52" s="3"/>
-      <c r="AP52" s="28"/>
-    </row>
-    <row r="53" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="D53" s="25"/>
-      <c r="L53" s="33"/>
-      <c r="M53" s="37"/>
-      <c r="N53" s="40"/>
-      <c r="P53" s="40"/>
-      <c r="Q53" s="45"/>
-      <c r="R53" s="26"/>
-      <c r="S53" s="26"/>
-      <c r="T53" s="26"/>
-      <c r="V53" s="3"/>
-      <c r="X53" s="3"/>
-      <c r="Z53" s="40"/>
-      <c r="AN53" s="3"/>
-      <c r="AP53" s="28"/>
-    </row>
-    <row r="54" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="D54" s="25"/>
-      <c r="L54" s="33"/>
-      <c r="M54" s="37"/>
-      <c r="N54" s="40"/>
-      <c r="P54" s="40"/>
-      <c r="Q54" s="45"/>
-      <c r="R54" s="26"/>
-      <c r="S54" s="26"/>
-      <c r="T54" s="26"/>
-      <c r="V54" s="3"/>
-      <c r="X54" s="3"/>
-      <c r="Z54" s="40"/>
-      <c r="AN54" s="3"/>
-      <c r="AP54" s="28"/>
-    </row>
-    <row r="55" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="D55" s="25"/>
-      <c r="L55" s="33"/>
-      <c r="M55" s="37"/>
-      <c r="N55" s="40"/>
-      <c r="P55" s="40"/>
-      <c r="Q55" s="45"/>
-      <c r="R55" s="26"/>
-      <c r="S55" s="26"/>
-      <c r="T55" s="26"/>
-      <c r="V55" s="3"/>
-      <c r="X55" s="3"/>
-      <c r="Z55" s="40"/>
-      <c r="AN55" s="3"/>
-      <c r="AP55" s="28"/>
-    </row>
-    <row r="56" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="D56" s="25"/>
-      <c r="L56" s="33"/>
-      <c r="M56" s="37"/>
-      <c r="N56" s="40"/>
-      <c r="P56" s="40"/>
-      <c r="Q56" s="45"/>
-      <c r="R56" s="26"/>
-      <c r="S56" s="26"/>
-      <c r="T56" s="26"/>
-      <c r="V56" s="3"/>
-      <c r="X56" s="3"/>
-      <c r="Z56" s="40"/>
-      <c r="AN56" s="3"/>
-      <c r="AP56" s="28"/>
-    </row>
-    <row r="57" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="D57" s="25"/>
-      <c r="L57" s="33"/>
-      <c r="M57" s="37"/>
-      <c r="N57" s="40"/>
-      <c r="P57" s="40"/>
-      <c r="Q57" s="45"/>
-      <c r="R57" s="26"/>
-      <c r="S57" s="26"/>
-      <c r="T57" s="26"/>
-      <c r="V57" s="3"/>
-      <c r="X57" s="3"/>
-      <c r="Z57" s="40"/>
-      <c r="AN57" s="3"/>
-      <c r="AP57" s="28"/>
-    </row>
-    <row r="58" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="D58" s="25"/>
-      <c r="L58" s="33"/>
-      <c r="M58" s="37"/>
-      <c r="N58" s="40"/>
-      <c r="P58" s="40"/>
-      <c r="Q58" s="45"/>
-      <c r="R58" s="26"/>
-      <c r="S58" s="26"/>
-      <c r="T58" s="26"/>
-      <c r="V58" s="3"/>
-      <c r="X58" s="3"/>
-      <c r="Z58" s="40"/>
-      <c r="AN58" s="3"/>
-      <c r="AP58" s="28"/>
-    </row>
-    <row r="59" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="D59" s="25"/>
-      <c r="L59" s="33"/>
-      <c r="M59" s="37"/>
-      <c r="N59" s="40"/>
-      <c r="P59" s="40"/>
-      <c r="Q59" s="45"/>
-      <c r="R59" s="26"/>
-      <c r="S59" s="26"/>
-      <c r="T59" s="26"/>
-      <c r="V59" s="3"/>
-      <c r="X59" s="3"/>
-      <c r="Z59" s="40"/>
-      <c r="AN59" s="3"/>
-      <c r="AP59" s="28"/>
-    </row>
-    <row r="60" spans="1:42" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="D60" s="25"/>
-      <c r="L60" s="33"/>
-      <c r="M60" s="37"/>
-      <c r="N60" s="40"/>
-      <c r="P60" s="40"/>
-      <c r="Q60" s="45"/>
-      <c r="R60" s="26"/>
-      <c r="S60" s="26"/>
-      <c r="T60" s="26"/>
-      <c r="V60" s="3"/>
-      <c r="X60" s="3"/>
-      <c r="Z60" s="40"/>
-      <c r="AN60" s="3"/>
-      <c r="AP60" s="28"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>